<commit_message>
Repair OT-1844 W012 cutoff review workbook v3 formatting
</commit_message>
<xml_diff>
--- a/projects/OT-1844/docs/schedule/OT1844_W012_revision_avance_corte_2026-03-15_v3.xlsx
+++ b/projects/OT-1844/docs/schedule/OT1844_W012_revision_avance_corte_2026-03-15_v3.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Revision_Avance_W012" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Revision_Avance_W012'!$A$1:$T$103</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -73,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -87,6 +89,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -481,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U103"/>
+  <dimension ref="A1:T103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -507,107 +512,106 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Entrega</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="11" t="inlineStr">
         <is>
           <t>Despacho/Tag</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="11" t="inlineStr">
         <is>
           <t>WBS</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="11" t="inlineStr">
         <is>
           <t>Actividad ID</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="11" t="inlineStr">
         <is>
           <t>Actividad</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Estado P6</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="11" t="inlineStr">
         <is>
           <t>Inicio Plan</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="11" t="inlineStr">
         <is>
           <t>Fin Plan</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Inicio Real</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Fin Real</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>% Complete Type</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>Calendar ID</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="11" t="inlineStr">
         <is>
           <t>Calendario</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>BAC HH</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>EV HH</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>ETC HH</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
         <is>
           <t>Avance acumulado corte %</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="11" t="inlineStr">
         <is>
           <t>% avance a cargar</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="11" t="inlineStr">
         <is>
           <t>Fecha inicio real a cargar</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="11" t="inlineStr">
         <is>
           <t>Fecha término si 100%</t>
         </is>
       </c>
-      <c r="U1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -685,8 +689,9 @@
       <c r="Q2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R2" s="2" t="inlineStr"/>
-      <c r="T2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -764,8 +769,9 @@
       <c r="Q3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R3" s="2" t="inlineStr"/>
-      <c r="T3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -843,8 +849,9 @@
       <c r="Q4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R4" s="2" t="inlineStr"/>
-      <c r="T4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -922,8 +929,9 @@
       <c r="Q5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R5" s="2" t="inlineStr"/>
-      <c r="T5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1001,8 +1009,9 @@
       <c r="Q6" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R6" s="2" t="inlineStr"/>
-      <c r="T6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1050,7 +1059,7 @@
           <t>2026-02-20 09:48:00</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -1076,8 +1085,9 @@
       <c r="Q7" s="7" t="n">
         <v>0.75</v>
       </c>
-      <c r="R7" s="5" t="inlineStr"/>
-      <c r="T7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="n"/>
+      <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1155,8 +1165,9 @@
       <c r="Q8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R8" s="2" t="inlineStr"/>
-      <c r="T8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1234,8 +1245,9 @@
       <c r="Q9" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R9" s="2" t="inlineStr"/>
-      <c r="T9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1313,8 +1325,9 @@
       <c r="Q10" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R10" s="2" t="inlineStr"/>
-      <c r="T10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="n"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1392,8 +1405,9 @@
       <c r="Q11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R11" s="2" t="inlineStr"/>
-      <c r="T11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1471,8 +1485,9 @@
       <c r="Q12" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R12" s="2" t="inlineStr"/>
-      <c r="T12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1550,8 +1565,9 @@
       <c r="Q13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="n"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1629,8 +1645,9 @@
       <c r="Q14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="n"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1708,8 +1725,9 @@
       <c r="Q15" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R15" s="2" t="inlineStr"/>
-      <c r="T15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="n"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1787,8 +1805,9 @@
       <c r="Q16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R16" s="2" t="inlineStr"/>
-      <c r="T16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="n"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1836,7 +1855,7 @@
           <t>2026-02-24 08:00:00</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="n"/>
       <c r="K17" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -1862,8 +1881,9 @@
       <c r="Q17" s="7" t="n">
         <v>0.75</v>
       </c>
-      <c r="R17" s="5" t="inlineStr"/>
-      <c r="T17" s="5" t="inlineStr"/>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="5" t="inlineStr"/>
+      <c r="T17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1911,7 +1931,7 @@
           <t>2026-02-23 08:00:00</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="n"/>
       <c r="K18" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -1937,8 +1957,9 @@
       <c r="Q18" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R18" s="5" t="inlineStr"/>
-      <c r="T18" s="5" t="inlineStr"/>
+      <c r="R18" s="5" t="n"/>
+      <c r="S18" s="5" t="inlineStr"/>
+      <c r="T18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2016,8 +2037,9 @@
       <c r="Q19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2095,8 +2117,9 @@
       <c r="Q20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="n"/>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2174,8 +2197,9 @@
       <c r="Q21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R21" s="2" t="inlineStr"/>
-      <c r="T21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="n"/>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -2223,7 +2247,7 @@
           <t>2026-02-24 16:12:00</t>
         </is>
       </c>
-      <c r="J22" s="5" t="inlineStr"/>
+      <c r="J22" s="5" t="n"/>
       <c r="K22" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2249,8 +2273,9 @@
       <c r="Q22" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R22" s="5" t="inlineStr"/>
-      <c r="T22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="n"/>
+      <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -2298,7 +2323,7 @@
           <t>2026-02-24 16:12:00</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr"/>
+      <c r="J23" s="5" t="n"/>
       <c r="K23" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2324,8 +2349,9 @@
       <c r="Q23" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R23" s="5" t="inlineStr"/>
-      <c r="T23" s="5" t="inlineStr"/>
+      <c r="R23" s="5" t="n"/>
+      <c r="S23" s="5" t="inlineStr"/>
+      <c r="T23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -2373,7 +2399,7 @@
           <t>2026-02-24 16:12:00</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr"/>
+      <c r="J24" s="5" t="n"/>
       <c r="K24" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2399,8 +2425,9 @@
       <c r="Q24" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R24" s="5" t="inlineStr"/>
-      <c r="T24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="n"/>
+      <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -2448,7 +2475,7 @@
           <t>2026-02-23 16:12:00</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="n"/>
       <c r="K25" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2474,8 +2501,9 @@
       <c r="Q25" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R25" s="5" t="inlineStr"/>
-      <c r="T25" s="5" t="inlineStr"/>
+      <c r="R25" s="5" t="n"/>
+      <c r="S25" s="5" t="inlineStr"/>
+      <c r="T25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2553,8 +2581,9 @@
       <c r="Q26" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R26" s="2" t="inlineStr"/>
-      <c r="T26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="n"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2632,8 +2661,9 @@
       <c r="Q27" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R27" s="2" t="inlineStr"/>
-      <c r="T27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="n"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -2681,7 +2711,7 @@
           <t>2026-02-26 16:12:00</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr"/>
+      <c r="J28" s="5" t="n"/>
       <c r="K28" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2707,8 +2737,9 @@
       <c r="Q28" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R28" s="5" t="inlineStr"/>
-      <c r="T28" s="5" t="inlineStr"/>
+      <c r="R28" s="5" t="n"/>
+      <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2756,7 +2787,7 @@
           <t>2026-02-25 16:12:00</t>
         </is>
       </c>
-      <c r="J29" s="5" t="inlineStr"/>
+      <c r="J29" s="5" t="n"/>
       <c r="K29" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2782,8 +2813,9 @@
       <c r="Q29" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R29" s="5" t="inlineStr"/>
-      <c r="T29" s="5" t="inlineStr"/>
+      <c r="R29" s="5" t="n"/>
+      <c r="S29" s="5" t="inlineStr"/>
+      <c r="T29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2831,7 +2863,7 @@
           <t>2026-02-27 16:12:00</t>
         </is>
       </c>
-      <c r="J30" s="5" t="inlineStr"/>
+      <c r="J30" s="5" t="n"/>
       <c r="K30" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2857,8 +2889,9 @@
       <c r="Q30" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="R30" s="5" t="inlineStr"/>
-      <c r="T30" s="5" t="inlineStr"/>
+      <c r="R30" s="5" t="n"/>
+      <c r="S30" s="5" t="inlineStr"/>
+      <c r="T30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2906,7 +2939,7 @@
           <t>2026-02-24 16:12:00</t>
         </is>
       </c>
-      <c r="J31" s="5" t="inlineStr"/>
+      <c r="J31" s="5" t="n"/>
       <c r="K31" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -2932,8 +2965,9 @@
       <c r="Q31" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R31" s="5" t="inlineStr"/>
-      <c r="T31" s="5" t="inlineStr"/>
+      <c r="R31" s="5" t="n"/>
+      <c r="S31" s="5" t="inlineStr"/>
+      <c r="T31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3011,8 +3045,9 @@
       <c r="Q32" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R32" s="2" t="inlineStr"/>
-      <c r="T32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="n"/>
+      <c r="S32" s="2" t="inlineStr"/>
+      <c r="T32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3090,8 +3125,9 @@
       <c r="Q33" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R33" s="2" t="inlineStr"/>
-      <c r="T33" s="2" t="inlineStr"/>
+      <c r="R33" s="2" t="n"/>
+      <c r="S33" s="2" t="inlineStr"/>
+      <c r="T33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3169,8 +3205,9 @@
       <c r="Q34" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R34" s="2" t="inlineStr"/>
-      <c r="T34" s="2" t="inlineStr"/>
+      <c r="R34" s="2" t="n"/>
+      <c r="S34" s="2" t="inlineStr"/>
+      <c r="T34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3218,7 +3255,7 @@
           <t>2026-02-27 14:24:00</t>
         </is>
       </c>
-      <c r="J35" s="5" t="inlineStr"/>
+      <c r="J35" s="5" t="n"/>
       <c r="K35" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -3244,8 +3281,9 @@
       <c r="Q35" s="7" t="n">
         <v>0.3</v>
       </c>
-      <c r="R35" s="5" t="inlineStr"/>
-      <c r="T35" s="5" t="inlineStr"/>
+      <c r="R35" s="5" t="n"/>
+      <c r="S35" s="5" t="inlineStr"/>
+      <c r="T35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3323,8 +3361,9 @@
       <c r="Q36" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R36" s="2" t="inlineStr"/>
-      <c r="T36" s="2" t="inlineStr"/>
+      <c r="R36" s="2" t="n"/>
+      <c r="S36" s="2" t="inlineStr"/>
+      <c r="T36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3402,8 +3441,9 @@
       <c r="Q37" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R37" s="2" t="inlineStr"/>
-      <c r="T37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="n"/>
+      <c r="S37" s="2" t="inlineStr"/>
+      <c r="T37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3481,8 +3521,9 @@
       <c r="Q38" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R38" s="2" t="inlineStr"/>
-      <c r="T38" s="2" t="inlineStr"/>
+      <c r="R38" s="2" t="n"/>
+      <c r="S38" s="2" t="inlineStr"/>
+      <c r="T38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -3530,7 +3571,7 @@
           <t>2026-03-08 08:00:00</t>
         </is>
       </c>
-      <c r="J39" s="5" t="inlineStr"/>
+      <c r="J39" s="5" t="n"/>
       <c r="K39" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -3556,8 +3597,9 @@
       <c r="Q39" s="7" t="n">
         <v>0.15</v>
       </c>
-      <c r="R39" s="5" t="inlineStr"/>
-      <c r="T39" s="5" t="inlineStr"/>
+      <c r="R39" s="5" t="n"/>
+      <c r="S39" s="5" t="inlineStr"/>
+      <c r="T39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -3605,7 +3647,7 @@
           <t>2026-03-06 08:00:00</t>
         </is>
       </c>
-      <c r="J40" s="5" t="inlineStr"/>
+      <c r="J40" s="5" t="n"/>
       <c r="K40" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -3631,8 +3673,9 @@
       <c r="Q40" s="7" t="n">
         <v>0.7</v>
       </c>
-      <c r="R40" s="5" t="inlineStr"/>
-      <c r="T40" s="5" t="inlineStr"/>
+      <c r="R40" s="5" t="n"/>
+      <c r="S40" s="5" t="inlineStr"/>
+      <c r="T40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3710,8 +3753,9 @@
       <c r="Q41" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R41" s="2" t="inlineStr"/>
-      <c r="T41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="n"/>
+      <c r="S41" s="2" t="inlineStr"/>
+      <c r="T41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3789,8 +3833,9 @@
       <c r="Q42" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R42" s="2" t="inlineStr"/>
-      <c r="T42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="n"/>
+      <c r="S42" s="2" t="inlineStr"/>
+      <c r="T42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
@@ -3833,8 +3878,8 @@
           <t>2026-03-09 18:00:00</t>
         </is>
       </c>
-      <c r="I43" s="8" t="inlineStr"/>
-      <c r="J43" s="8" t="inlineStr"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -3860,8 +3905,9 @@
       <c r="Q43" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R43" s="8" t="inlineStr"/>
-      <c r="T43" s="8" t="inlineStr"/>
+      <c r="R43" s="8" t="n"/>
+      <c r="S43" s="8" t="inlineStr"/>
+      <c r="T43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3939,8 +3985,9 @@
       <c r="Q44" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R44" s="2" t="inlineStr"/>
-      <c r="T44" s="2" t="inlineStr"/>
+      <c r="R44" s="2" t="n"/>
+      <c r="S44" s="2" t="inlineStr"/>
+      <c r="T44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
@@ -3988,7 +4035,7 @@
           <t>2026-03-07 08:00:00</t>
         </is>
       </c>
-      <c r="J45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="n"/>
       <c r="K45" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4014,8 +4061,9 @@
       <c r="Q45" s="7" t="n">
         <v>0.5</v>
       </c>
-      <c r="R45" s="5" t="inlineStr"/>
-      <c r="T45" s="5" t="inlineStr"/>
+      <c r="R45" s="5" t="n"/>
+      <c r="S45" s="5" t="inlineStr"/>
+      <c r="T45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -4058,8 +4106,8 @@
           <t>2026-03-10 18:00:00</t>
         </is>
       </c>
-      <c r="I46" s="8" t="inlineStr"/>
-      <c r="J46" s="8" t="inlineStr"/>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8" t="n"/>
       <c r="K46" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4085,8 +4133,9 @@
       <c r="Q46" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R46" s="8" t="inlineStr"/>
-      <c r="T46" s="8" t="inlineStr"/>
+      <c r="R46" s="8" t="n"/>
+      <c r="S46" s="8" t="inlineStr"/>
+      <c r="T46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4164,8 +4213,9 @@
       <c r="Q47" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R47" s="2" t="inlineStr"/>
-      <c r="T47" s="2" t="inlineStr"/>
+      <c r="R47" s="2" t="n"/>
+      <c r="S47" s="2" t="inlineStr"/>
+      <c r="T47" s="2" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -4208,8 +4258,8 @@
           <t>2026-03-11 18:00:00</t>
         </is>
       </c>
-      <c r="I48" s="8" t="inlineStr"/>
-      <c r="J48" s="8" t="inlineStr"/>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8" t="n"/>
       <c r="K48" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4235,8 +4285,9 @@
       <c r="Q48" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R48" s="8" t="inlineStr"/>
-      <c r="T48" s="8" t="inlineStr"/>
+      <c r="R48" s="8" t="n"/>
+      <c r="S48" s="8" t="inlineStr"/>
+      <c r="T48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4314,8 +4365,9 @@
       <c r="Q49" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R49" s="2" t="inlineStr"/>
-      <c r="T49" s="2" t="inlineStr"/>
+      <c r="R49" s="2" t="n"/>
+      <c r="S49" s="2" t="inlineStr"/>
+      <c r="T49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -4358,8 +4410,8 @@
           <t>2026-03-11 18:00:00</t>
         </is>
       </c>
-      <c r="I50" s="8" t="inlineStr"/>
-      <c r="J50" s="8" t="inlineStr"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
       <c r="K50" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4385,8 +4437,9 @@
       <c r="Q50" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R50" s="8" t="inlineStr"/>
-      <c r="T50" s="8" t="inlineStr"/>
+      <c r="R50" s="8" t="n"/>
+      <c r="S50" s="8" t="inlineStr"/>
+      <c r="T50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4464,8 +4517,9 @@
       <c r="Q51" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R51" s="2" t="inlineStr"/>
-      <c r="T51" s="2" t="inlineStr"/>
+      <c r="R51" s="2" t="n"/>
+      <c r="S51" s="2" t="inlineStr"/>
+      <c r="T51" s="2" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -4508,8 +4562,8 @@
           <t>2026-03-11 18:00:00</t>
         </is>
       </c>
-      <c r="I52" s="8" t="inlineStr"/>
-      <c r="J52" s="8" t="inlineStr"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="J52" s="8" t="n"/>
       <c r="K52" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4535,8 +4589,9 @@
       <c r="Q52" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R52" s="8" t="inlineStr"/>
-      <c r="T52" s="8" t="inlineStr"/>
+      <c r="R52" s="8" t="n"/>
+      <c r="S52" s="8" t="inlineStr"/>
+      <c r="T52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4614,8 +4669,9 @@
       <c r="Q53" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R53" s="2" t="inlineStr"/>
-      <c r="T53" s="2" t="inlineStr"/>
+      <c r="R53" s="2" t="n"/>
+      <c r="S53" s="2" t="inlineStr"/>
+      <c r="T53" s="2" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -4658,8 +4714,8 @@
           <t>2026-03-11 18:00:00</t>
         </is>
       </c>
-      <c r="I54" s="8" t="inlineStr"/>
-      <c r="J54" s="8" t="inlineStr"/>
+      <c r="I54" s="8" t="n"/>
+      <c r="J54" s="8" t="n"/>
       <c r="K54" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4685,8 +4741,9 @@
       <c r="Q54" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R54" s="8" t="inlineStr"/>
-      <c r="T54" s="8" t="inlineStr"/>
+      <c r="R54" s="8" t="n"/>
+      <c r="S54" s="8" t="inlineStr"/>
+      <c r="T54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -4729,8 +4786,8 @@
           <t>2026-03-10 11:36:00</t>
         </is>
       </c>
-      <c r="I55" s="8" t="inlineStr"/>
-      <c r="J55" s="8" t="inlineStr"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
       <c r="K55" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4756,8 +4813,9 @@
       <c r="Q55" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R55" s="8" t="inlineStr"/>
-      <c r="T55" s="8" t="inlineStr"/>
+      <c r="R55" s="8" t="n"/>
+      <c r="S55" s="8" t="inlineStr"/>
+      <c r="T55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -4800,8 +4858,8 @@
           <t>2026-03-10 11:36:00</t>
         </is>
       </c>
-      <c r="I56" s="8" t="inlineStr"/>
-      <c r="J56" s="8" t="inlineStr"/>
+      <c r="I56" s="8" t="n"/>
+      <c r="J56" s="8" t="n"/>
       <c r="K56" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4827,8 +4885,9 @@
       <c r="Q56" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R56" s="8" t="inlineStr"/>
-      <c r="T56" s="8" t="inlineStr"/>
+      <c r="R56" s="8" t="n"/>
+      <c r="S56" s="8" t="inlineStr"/>
+      <c r="T56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
@@ -4871,8 +4930,8 @@
           <t>2026-03-11 14:24:00</t>
         </is>
       </c>
-      <c r="I57" s="8" t="inlineStr"/>
-      <c r="J57" s="8" t="inlineStr"/>
+      <c r="I57" s="8" t="n"/>
+      <c r="J57" s="8" t="n"/>
       <c r="K57" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4898,8 +4957,9 @@
       <c r="Q57" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R57" s="8" t="inlineStr"/>
-      <c r="T57" s="8" t="inlineStr"/>
+      <c r="R57" s="8" t="n"/>
+      <c r="S57" s="8" t="inlineStr"/>
+      <c r="T57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -4942,8 +5002,8 @@
           <t>2026-03-10 18:00:00</t>
         </is>
       </c>
-      <c r="I58" s="8" t="inlineStr"/>
-      <c r="J58" s="8" t="inlineStr"/>
+      <c r="I58" s="8" t="n"/>
+      <c r="J58" s="8" t="n"/>
       <c r="K58" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -4969,8 +5029,9 @@
       <c r="Q58" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R58" s="8" t="inlineStr"/>
-      <c r="T58" s="8" t="inlineStr"/>
+      <c r="R58" s="8" t="n"/>
+      <c r="S58" s="8" t="inlineStr"/>
+      <c r="T58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -5013,8 +5074,8 @@
           <t>2026-03-10 18:00:00</t>
         </is>
       </c>
-      <c r="I59" s="8" t="inlineStr"/>
-      <c r="J59" s="8" t="inlineStr"/>
+      <c r="I59" s="8" t="n"/>
+      <c r="J59" s="8" t="n"/>
       <c r="K59" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5040,8 +5101,9 @@
       <c r="Q59" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R59" s="8" t="inlineStr"/>
-      <c r="T59" s="8" t="inlineStr"/>
+      <c r="R59" s="8" t="n"/>
+      <c r="S59" s="8" t="inlineStr"/>
+      <c r="T59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5119,8 +5181,9 @@
       <c r="Q60" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R60" s="2" t="inlineStr"/>
-      <c r="T60" s="2" t="inlineStr"/>
+      <c r="R60" s="2" t="n"/>
+      <c r="S60" s="2" t="inlineStr"/>
+      <c r="T60" s="2" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -5163,8 +5226,8 @@
           <t>2026-03-11 11:36:00</t>
         </is>
       </c>
-      <c r="I61" s="8" t="inlineStr"/>
-      <c r="J61" s="8" t="inlineStr"/>
+      <c r="I61" s="8" t="n"/>
+      <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5190,8 +5253,9 @@
       <c r="Q61" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R61" s="8" t="inlineStr"/>
-      <c r="T61" s="8" t="inlineStr"/>
+      <c r="R61" s="8" t="n"/>
+      <c r="S61" s="8" t="inlineStr"/>
+      <c r="T61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
@@ -5234,8 +5298,8 @@
           <t>2026-03-11 11:36:00</t>
         </is>
       </c>
-      <c r="I62" s="8" t="inlineStr"/>
-      <c r="J62" s="8" t="inlineStr"/>
+      <c r="I62" s="8" t="n"/>
+      <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5261,8 +5325,9 @@
       <c r="Q62" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R62" s="8" t="inlineStr"/>
-      <c r="T62" s="8" t="inlineStr"/>
+      <c r="R62" s="8" t="n"/>
+      <c r="S62" s="8" t="inlineStr"/>
+      <c r="T62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
@@ -5305,8 +5370,8 @@
           <t>2026-03-11 12:57:00</t>
         </is>
       </c>
-      <c r="I63" s="8" t="inlineStr"/>
-      <c r="J63" s="8" t="inlineStr"/>
+      <c r="I63" s="8" t="n"/>
+      <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5332,8 +5397,9 @@
       <c r="Q63" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R63" s="8" t="inlineStr"/>
-      <c r="T63" s="8" t="inlineStr"/>
+      <c r="R63" s="8" t="n"/>
+      <c r="S63" s="8" t="inlineStr"/>
+      <c r="T63" s="8" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
@@ -5376,8 +5442,8 @@
           <t>2026-03-11 14:24:00</t>
         </is>
       </c>
-      <c r="I64" s="8" t="inlineStr"/>
-      <c r="J64" s="8" t="inlineStr"/>
+      <c r="I64" s="8" t="n"/>
+      <c r="J64" s="8" t="n"/>
       <c r="K64" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5403,8 +5469,9 @@
       <c r="Q64" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R64" s="8" t="inlineStr"/>
-      <c r="T64" s="8" t="inlineStr"/>
+      <c r="R64" s="8" t="n"/>
+      <c r="S64" s="8" t="inlineStr"/>
+      <c r="T64" s="8" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
@@ -5447,8 +5514,8 @@
           <t>2026-03-13 15:45:00</t>
         </is>
       </c>
-      <c r="I65" s="8" t="inlineStr"/>
-      <c r="J65" s="8" t="inlineStr"/>
+      <c r="I65" s="8" t="n"/>
+      <c r="J65" s="8" t="n"/>
       <c r="K65" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5474,8 +5541,9 @@
       <c r="Q65" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R65" s="8" t="inlineStr"/>
-      <c r="T65" s="8" t="inlineStr"/>
+      <c r="R65" s="8" t="n"/>
+      <c r="S65" s="8" t="inlineStr"/>
+      <c r="T65" s="8" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
@@ -5518,8 +5586,8 @@
           <t>2026-03-11 18:00:00</t>
         </is>
       </c>
-      <c r="I66" s="8" t="inlineStr"/>
-      <c r="J66" s="8" t="inlineStr"/>
+      <c r="I66" s="8" t="n"/>
+      <c r="J66" s="8" t="n"/>
       <c r="K66" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5545,8 +5613,9 @@
       <c r="Q66" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R66" s="8" t="inlineStr"/>
-      <c r="T66" s="8" t="inlineStr"/>
+      <c r="R66" s="8" t="n"/>
+      <c r="S66" s="8" t="inlineStr"/>
+      <c r="T66" s="8" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5624,8 +5693,9 @@
       <c r="Q67" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R67" s="2" t="inlineStr"/>
-      <c r="T67" s="2" t="inlineStr"/>
+      <c r="R67" s="2" t="n"/>
+      <c r="S67" s="2" t="inlineStr"/>
+      <c r="T67" s="2" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
@@ -5668,8 +5738,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I68" s="8" t="inlineStr"/>
-      <c r="J68" s="8" t="inlineStr"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="8" t="n"/>
       <c r="K68" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5695,8 +5765,9 @@
       <c r="Q68" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R68" s="8" t="inlineStr"/>
-      <c r="T68" s="8" t="inlineStr"/>
+      <c r="R68" s="8" t="n"/>
+      <c r="S68" s="8" t="inlineStr"/>
+      <c r="T68" s="8" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
@@ -5744,7 +5815,7 @@
           <t>2026-03-05 08:00:00</t>
         </is>
       </c>
-      <c r="J69" s="5" t="inlineStr"/>
+      <c r="J69" s="5" t="n"/>
       <c r="K69" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5770,8 +5841,9 @@
       <c r="Q69" s="7" t="n">
         <v>0.8</v>
       </c>
-      <c r="R69" s="5" t="inlineStr"/>
-      <c r="T69" s="5" t="inlineStr"/>
+      <c r="R69" s="5" t="n"/>
+      <c r="S69" s="5" t="inlineStr"/>
+      <c r="T69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5849,8 +5921,9 @@
       <c r="Q70" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R70" s="2" t="inlineStr"/>
-      <c r="T70" s="2" t="inlineStr"/>
+      <c r="R70" s="2" t="n"/>
+      <c r="S70" s="2" t="inlineStr"/>
+      <c r="T70" s="2" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
@@ -5893,8 +5966,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I71" s="8" t="inlineStr"/>
-      <c r="J71" s="8" t="inlineStr"/>
+      <c r="I71" s="8" t="n"/>
+      <c r="J71" s="8" t="n"/>
       <c r="K71" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5920,8 +5993,9 @@
       <c r="Q71" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R71" s="8" t="inlineStr"/>
-      <c r="T71" s="8" t="inlineStr"/>
+      <c r="R71" s="8" t="n"/>
+      <c r="S71" s="8" t="inlineStr"/>
+      <c r="T71" s="8" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
@@ -5964,8 +6038,8 @@
           <t>2026-03-12 09:48:00</t>
         </is>
       </c>
-      <c r="I72" s="8" t="inlineStr"/>
-      <c r="J72" s="8" t="inlineStr"/>
+      <c r="I72" s="8" t="n"/>
+      <c r="J72" s="8" t="n"/>
       <c r="K72" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -5991,8 +6065,9 @@
       <c r="Q72" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R72" s="8" t="inlineStr"/>
-      <c r="T72" s="8" t="inlineStr"/>
+      <c r="R72" s="8" t="n"/>
+      <c r="S72" s="8" t="inlineStr"/>
+      <c r="T72" s="8" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="inlineStr">
@@ -6035,8 +6110,8 @@
           <t>2026-03-12 11:36:00</t>
         </is>
       </c>
-      <c r="I73" s="8" t="inlineStr"/>
-      <c r="J73" s="8" t="inlineStr"/>
+      <c r="I73" s="8" t="n"/>
+      <c r="J73" s="8" t="n"/>
       <c r="K73" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6062,8 +6137,9 @@
       <c r="Q73" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R73" s="8" t="inlineStr"/>
-      <c r="T73" s="8" t="inlineStr"/>
+      <c r="R73" s="8" t="n"/>
+      <c r="S73" s="8" t="inlineStr"/>
+      <c r="T73" s="8" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="8" t="inlineStr">
@@ -6106,8 +6182,8 @@
           <t>2026-03-12 11:36:00</t>
         </is>
       </c>
-      <c r="I74" s="8" t="inlineStr"/>
-      <c r="J74" s="8" t="inlineStr"/>
+      <c r="I74" s="8" t="n"/>
+      <c r="J74" s="8" t="n"/>
       <c r="K74" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6133,8 +6209,9 @@
       <c r="Q74" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R74" s="8" t="inlineStr"/>
-      <c r="T74" s="8" t="inlineStr"/>
+      <c r="R74" s="8" t="n"/>
+      <c r="S74" s="8" t="inlineStr"/>
+      <c r="T74" s="8" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
@@ -6177,8 +6254,8 @@
           <t>2026-03-12 11:36:00</t>
         </is>
       </c>
-      <c r="I75" s="8" t="inlineStr"/>
-      <c r="J75" s="8" t="inlineStr"/>
+      <c r="I75" s="8" t="n"/>
+      <c r="J75" s="8" t="n"/>
       <c r="K75" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6204,8 +6281,9 @@
       <c r="Q75" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R75" s="8" t="inlineStr"/>
-      <c r="T75" s="8" t="inlineStr"/>
+      <c r="R75" s="8" t="n"/>
+      <c r="S75" s="8" t="inlineStr"/>
+      <c r="T75" s="8" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
@@ -6248,8 +6326,8 @@
           <t>2026-03-14 12:30:00</t>
         </is>
       </c>
-      <c r="I76" s="8" t="inlineStr"/>
-      <c r="J76" s="8" t="inlineStr"/>
+      <c r="I76" s="8" t="n"/>
+      <c r="J76" s="8" t="n"/>
       <c r="K76" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6275,8 +6353,9 @@
       <c r="Q76" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R76" s="8" t="inlineStr"/>
-      <c r="T76" s="8" t="inlineStr"/>
+      <c r="R76" s="8" t="n"/>
+      <c r="S76" s="8" t="inlineStr"/>
+      <c r="T76" s="8" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -6324,7 +6403,7 @@
           <t>2026-03-07 14:24:00</t>
         </is>
       </c>
-      <c r="J77" s="5" t="inlineStr"/>
+      <c r="J77" s="5" t="n"/>
       <c r="K77" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6350,8 +6429,9 @@
       <c r="Q77" s="7" t="n">
         <v>0.2</v>
       </c>
-      <c r="R77" s="5" t="inlineStr"/>
-      <c r="T77" s="5" t="inlineStr"/>
+      <c r="R77" s="5" t="n"/>
+      <c r="S77" s="5" t="inlineStr"/>
+      <c r="T77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -6399,7 +6479,7 @@
           <t>2026-03-02 08:00:00</t>
         </is>
       </c>
-      <c r="J78" s="5" t="inlineStr"/>
+      <c r="J78" s="5" t="n"/>
       <c r="K78" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6425,8 +6505,9 @@
       <c r="Q78" s="7" t="n">
         <v>0.6</v>
       </c>
-      <c r="R78" s="5" t="inlineStr"/>
-      <c r="T78" s="5" t="inlineStr"/>
+      <c r="R78" s="5" t="n"/>
+      <c r="S78" s="5" t="inlineStr"/>
+      <c r="T78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
@@ -6469,8 +6550,8 @@
           <t>2026-03-14 18:00:00</t>
         </is>
       </c>
-      <c r="I79" s="8" t="inlineStr"/>
-      <c r="J79" s="8" t="inlineStr"/>
+      <c r="I79" s="8" t="n"/>
+      <c r="J79" s="8" t="n"/>
       <c r="K79" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6496,8 +6577,9 @@
       <c r="Q79" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R79" s="8" t="inlineStr"/>
-      <c r="T79" s="8" t="inlineStr"/>
+      <c r="R79" s="8" t="n"/>
+      <c r="S79" s="8" t="inlineStr"/>
+      <c r="T79" s="8" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="8" t="inlineStr">
@@ -6540,8 +6622,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I80" s="8" t="inlineStr"/>
-      <c r="J80" s="8" t="inlineStr"/>
+      <c r="I80" s="8" t="n"/>
+      <c r="J80" s="8" t="n"/>
       <c r="K80" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6567,8 +6649,9 @@
       <c r="Q80" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R80" s="8" t="inlineStr"/>
-      <c r="T80" s="8" t="inlineStr"/>
+      <c r="R80" s="8" t="n"/>
+      <c r="S80" s="8" t="inlineStr"/>
+      <c r="T80" s="8" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
@@ -6611,8 +6694,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I81" s="8" t="inlineStr"/>
-      <c r="J81" s="8" t="inlineStr"/>
+      <c r="I81" s="8" t="n"/>
+      <c r="J81" s="8" t="n"/>
       <c r="K81" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6638,8 +6721,9 @@
       <c r="Q81" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R81" s="8" t="inlineStr"/>
-      <c r="T81" s="8" t="inlineStr"/>
+      <c r="R81" s="8" t="n"/>
+      <c r="S81" s="8" t="inlineStr"/>
+      <c r="T81" s="8" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
@@ -6682,8 +6766,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I82" s="8" t="inlineStr"/>
-      <c r="J82" s="8" t="inlineStr"/>
+      <c r="I82" s="8" t="n"/>
+      <c r="J82" s="8" t="n"/>
       <c r="K82" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6709,8 +6793,9 @@
       <c r="Q82" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R82" s="8" t="inlineStr"/>
-      <c r="T82" s="8" t="inlineStr"/>
+      <c r="R82" s="8" t="n"/>
+      <c r="S82" s="8" t="inlineStr"/>
+      <c r="T82" s="8" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
@@ -6753,8 +6838,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I83" s="8" t="inlineStr"/>
-      <c r="J83" s="8" t="inlineStr"/>
+      <c r="I83" s="8" t="n"/>
+      <c r="J83" s="8" t="n"/>
       <c r="K83" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6780,8 +6865,9 @@
       <c r="Q83" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R83" s="8" t="inlineStr"/>
-      <c r="T83" s="8" t="inlineStr"/>
+      <c r="R83" s="8" t="n"/>
+      <c r="S83" s="8" t="inlineStr"/>
+      <c r="T83" s="8" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
@@ -6824,8 +6910,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I84" s="8" t="inlineStr"/>
-      <c r="J84" s="8" t="inlineStr"/>
+      <c r="I84" s="8" t="n"/>
+      <c r="J84" s="8" t="n"/>
       <c r="K84" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6851,8 +6937,9 @@
       <c r="Q84" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R84" s="8" t="inlineStr"/>
-      <c r="T84" s="8" t="inlineStr"/>
+      <c r="R84" s="8" t="n"/>
+      <c r="S84" s="8" t="inlineStr"/>
+      <c r="T84" s="8" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -6900,7 +6987,7 @@
           <t>2026-03-02 11:36:00</t>
         </is>
       </c>
-      <c r="J85" s="5" t="inlineStr"/>
+      <c r="J85" s="5" t="n"/>
       <c r="K85" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -6926,8 +7013,9 @@
       <c r="Q85" s="7" t="n">
         <v>0.6</v>
       </c>
-      <c r="R85" s="5" t="inlineStr"/>
-      <c r="T85" s="5" t="inlineStr"/>
+      <c r="R85" s="5" t="n"/>
+      <c r="S85" s="5" t="inlineStr"/>
+      <c r="T85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -6975,7 +7063,7 @@
           <t>2026-03-02 11:36:00</t>
         </is>
       </c>
-      <c r="J86" s="5" t="inlineStr"/>
+      <c r="J86" s="5" t="n"/>
       <c r="K86" s="5" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7001,8 +7089,9 @@
       <c r="Q86" s="7" t="n">
         <v>0.7</v>
       </c>
-      <c r="R86" s="5" t="inlineStr"/>
-      <c r="T86" s="5" t="inlineStr"/>
+      <c r="R86" s="5" t="n"/>
+      <c r="S86" s="5" t="inlineStr"/>
+      <c r="T86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="8" t="inlineStr">
@@ -7045,8 +7134,8 @@
           <t>2026-03-13 11:36:00</t>
         </is>
       </c>
-      <c r="I87" s="8" t="inlineStr"/>
-      <c r="J87" s="8" t="inlineStr"/>
+      <c r="I87" s="8" t="n"/>
+      <c r="J87" s="8" t="n"/>
       <c r="K87" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7072,8 +7161,9 @@
       <c r="Q87" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R87" s="8" t="inlineStr"/>
-      <c r="T87" s="8" t="inlineStr"/>
+      <c r="R87" s="8" t="n"/>
+      <c r="S87" s="8" t="inlineStr"/>
+      <c r="T87" s="8" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="8" t="inlineStr">
@@ -7116,8 +7206,8 @@
           <t>2026-03-15 12:00:00</t>
         </is>
       </c>
-      <c r="I88" s="8" t="inlineStr"/>
-      <c r="J88" s="8" t="inlineStr"/>
+      <c r="I88" s="8" t="n"/>
+      <c r="J88" s="8" t="n"/>
       <c r="K88" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7143,8 +7233,9 @@
       <c r="Q88" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R88" s="8" t="inlineStr"/>
-      <c r="T88" s="8" t="inlineStr"/>
+      <c r="R88" s="8" t="n"/>
+      <c r="S88" s="8" t="inlineStr"/>
+      <c r="T88" s="8" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="8" t="inlineStr">
@@ -7187,8 +7278,8 @@
           <t>2026-03-13 14:24:00</t>
         </is>
       </c>
-      <c r="I89" s="8" t="inlineStr"/>
-      <c r="J89" s="8" t="inlineStr"/>
+      <c r="I89" s="8" t="n"/>
+      <c r="J89" s="8" t="n"/>
       <c r="K89" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7214,8 +7305,9 @@
       <c r="Q89" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R89" s="8" t="inlineStr"/>
-      <c r="T89" s="8" t="inlineStr"/>
+      <c r="R89" s="8" t="n"/>
+      <c r="S89" s="8" t="inlineStr"/>
+      <c r="T89" s="8" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="8" t="inlineStr">
@@ -7258,8 +7350,8 @@
           <t>2026-03-13 15:45:00</t>
         </is>
       </c>
-      <c r="I90" s="8" t="inlineStr"/>
-      <c r="J90" s="8" t="inlineStr"/>
+      <c r="I90" s="8" t="n"/>
+      <c r="J90" s="8" t="n"/>
       <c r="K90" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7285,8 +7377,9 @@
       <c r="Q90" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R90" s="8" t="inlineStr"/>
-      <c r="T90" s="8" t="inlineStr"/>
+      <c r="R90" s="8" t="n"/>
+      <c r="S90" s="8" t="inlineStr"/>
+      <c r="T90" s="8" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="8" t="inlineStr">
@@ -7329,8 +7422,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I91" s="8" t="inlineStr"/>
-      <c r="J91" s="8" t="inlineStr"/>
+      <c r="I91" s="8" t="n"/>
+      <c r="J91" s="8" t="n"/>
       <c r="K91" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7356,8 +7449,9 @@
       <c r="Q91" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R91" s="8" t="inlineStr"/>
-      <c r="T91" s="8" t="inlineStr"/>
+      <c r="R91" s="8" t="n"/>
+      <c r="S91" s="8" t="inlineStr"/>
+      <c r="T91" s="8" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="8" t="inlineStr">
@@ -7400,8 +7494,8 @@
           <t>2026-03-13 18:00:00</t>
         </is>
       </c>
-      <c r="I92" s="8" t="inlineStr"/>
-      <c r="J92" s="8" t="inlineStr"/>
+      <c r="I92" s="8" t="n"/>
+      <c r="J92" s="8" t="n"/>
       <c r="K92" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7427,8 +7521,9 @@
       <c r="Q92" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R92" s="8" t="inlineStr"/>
-      <c r="T92" s="8" t="inlineStr"/>
+      <c r="R92" s="8" t="n"/>
+      <c r="S92" s="8" t="inlineStr"/>
+      <c r="T92" s="8" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="8" t="inlineStr">
@@ -7471,8 +7566,8 @@
           <t>2026-03-20 18:00:00</t>
         </is>
       </c>
-      <c r="I93" s="8" t="inlineStr"/>
-      <c r="J93" s="8" t="inlineStr"/>
+      <c r="I93" s="8" t="n"/>
+      <c r="J93" s="8" t="n"/>
       <c r="K93" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7498,8 +7593,9 @@
       <c r="Q93" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R93" s="8" t="inlineStr"/>
-      <c r="T93" s="8" t="inlineStr"/>
+      <c r="R93" s="8" t="n"/>
+      <c r="S93" s="8" t="inlineStr"/>
+      <c r="T93" s="8" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="8" t="inlineStr">
@@ -7542,8 +7638,8 @@
           <t>2026-03-16 18:00:00</t>
         </is>
       </c>
-      <c r="I94" s="8" t="inlineStr"/>
-      <c r="J94" s="8" t="inlineStr"/>
+      <c r="I94" s="8" t="n"/>
+      <c r="J94" s="8" t="n"/>
       <c r="K94" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7569,8 +7665,9 @@
       <c r="Q94" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R94" s="8" t="inlineStr"/>
-      <c r="T94" s="8" t="inlineStr"/>
+      <c r="R94" s="8" t="n"/>
+      <c r="S94" s="8" t="inlineStr"/>
+      <c r="T94" s="8" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="8" t="inlineStr">
@@ -7613,8 +7710,8 @@
           <t>2026-03-14 09:48:00</t>
         </is>
       </c>
-      <c r="I95" s="8" t="inlineStr"/>
-      <c r="J95" s="8" t="inlineStr"/>
+      <c r="I95" s="8" t="n"/>
+      <c r="J95" s="8" t="n"/>
       <c r="K95" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7640,8 +7737,9 @@
       <c r="Q95" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R95" s="8" t="inlineStr"/>
-      <c r="T95" s="8" t="inlineStr"/>
+      <c r="R95" s="8" t="n"/>
+      <c r="S95" s="8" t="inlineStr"/>
+      <c r="T95" s="8" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="8" t="inlineStr">
@@ -7684,8 +7782,8 @@
           <t>2026-03-16 10:42:00</t>
         </is>
       </c>
-      <c r="I96" s="8" t="inlineStr"/>
-      <c r="J96" s="8" t="inlineStr"/>
+      <c r="I96" s="8" t="n"/>
+      <c r="J96" s="8" t="n"/>
       <c r="K96" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7711,8 +7809,9 @@
       <c r="Q96" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R96" s="8" t="inlineStr"/>
-      <c r="T96" s="8" t="inlineStr"/>
+      <c r="R96" s="8" t="n"/>
+      <c r="S96" s="8" t="inlineStr"/>
+      <c r="T96" s="8" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="8" t="inlineStr">
@@ -7755,8 +7854,8 @@
           <t>2026-03-16 11:36:00</t>
         </is>
       </c>
-      <c r="I97" s="8" t="inlineStr"/>
-      <c r="J97" s="8" t="inlineStr"/>
+      <c r="I97" s="8" t="n"/>
+      <c r="J97" s="8" t="n"/>
       <c r="K97" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7782,8 +7881,9 @@
       <c r="Q97" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R97" s="8" t="inlineStr"/>
-      <c r="T97" s="8" t="inlineStr"/>
+      <c r="R97" s="8" t="n"/>
+      <c r="S97" s="8" t="inlineStr"/>
+      <c r="T97" s="8" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
@@ -7826,8 +7926,8 @@
           <t>2026-03-14 18:00:00</t>
         </is>
       </c>
-      <c r="I98" s="8" t="inlineStr"/>
-      <c r="J98" s="8" t="inlineStr"/>
+      <c r="I98" s="8" t="n"/>
+      <c r="J98" s="8" t="n"/>
       <c r="K98" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7853,8 +7953,9 @@
       <c r="Q98" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R98" s="8" t="inlineStr"/>
-      <c r="T98" s="8" t="inlineStr"/>
+      <c r="R98" s="8" t="n"/>
+      <c r="S98" s="8" t="inlineStr"/>
+      <c r="T98" s="8" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="8" t="inlineStr">
@@ -7897,8 +7998,8 @@
           <t>2026-03-14 18:00:00</t>
         </is>
       </c>
-      <c r="I99" s="8" t="inlineStr"/>
-      <c r="J99" s="8" t="inlineStr"/>
+      <c r="I99" s="8" t="n"/>
+      <c r="J99" s="8" t="n"/>
       <c r="K99" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7924,8 +8025,9 @@
       <c r="Q99" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R99" s="8" t="inlineStr"/>
-      <c r="T99" s="8" t="inlineStr"/>
+      <c r="R99" s="8" t="n"/>
+      <c r="S99" s="8" t="inlineStr"/>
+      <c r="T99" s="8" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="8" t="inlineStr">
@@ -7968,8 +8070,8 @@
           <t>2026-03-15 12:00:00</t>
         </is>
       </c>
-      <c r="I100" s="8" t="inlineStr"/>
-      <c r="J100" s="8" t="inlineStr"/>
+      <c r="I100" s="8" t="n"/>
+      <c r="J100" s="8" t="n"/>
       <c r="K100" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -7995,8 +8097,9 @@
       <c r="Q100" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R100" s="8" t="inlineStr"/>
-      <c r="T100" s="8" t="inlineStr"/>
+      <c r="R100" s="8" t="n"/>
+      <c r="S100" s="8" t="inlineStr"/>
+      <c r="T100" s="8" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="8" t="inlineStr">
@@ -8039,8 +8142,8 @@
           <t>2026-03-15 16:30:00</t>
         </is>
       </c>
-      <c r="I101" s="8" t="inlineStr"/>
-      <c r="J101" s="8" t="inlineStr"/>
+      <c r="I101" s="8" t="n"/>
+      <c r="J101" s="8" t="n"/>
       <c r="K101" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -8066,8 +8169,9 @@
       <c r="Q101" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R101" s="8" t="inlineStr"/>
-      <c r="T101" s="8" t="inlineStr"/>
+      <c r="R101" s="8" t="n"/>
+      <c r="S101" s="8" t="inlineStr"/>
+      <c r="T101" s="8" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="8" t="inlineStr">
@@ -8110,8 +8214,8 @@
           <t>2026-03-15 16:30:00</t>
         </is>
       </c>
-      <c r="I102" s="8" t="inlineStr"/>
-      <c r="J102" s="8" t="inlineStr"/>
+      <c r="I102" s="8" t="n"/>
+      <c r="J102" s="8" t="n"/>
       <c r="K102" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -8137,8 +8241,9 @@
       <c r="Q102" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R102" s="8" t="inlineStr"/>
-      <c r="T102" s="8" t="inlineStr"/>
+      <c r="R102" s="8" t="n"/>
+      <c r="S102" s="8" t="inlineStr"/>
+      <c r="T102" s="8" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="8" t="inlineStr">
@@ -8181,8 +8286,8 @@
           <t>2026-03-16 12:30:00</t>
         </is>
       </c>
-      <c r="I103" s="8" t="inlineStr"/>
-      <c r="J103" s="8" t="inlineStr"/>
+      <c r="I103" s="8" t="n"/>
+      <c r="J103" s="8" t="n"/>
       <c r="K103" s="8" t="inlineStr">
         <is>
           <t>CP_Drtn</t>
@@ -8208,10 +8313,12 @@
       <c r="Q103" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="R103" s="8" t="inlineStr"/>
-      <c r="T103" s="8" t="inlineStr"/>
+      <c r="R103" s="8" t="n"/>
+      <c r="S103" s="8" t="inlineStr"/>
+      <c r="T103" s="8" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:T103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>